<commit_message>
docs(tutorials): FEM-3 Part 3 re-locked on the rebuilt models and read from their strain fields
Fill c' = 5 kPa and a 4 m foundation for both pairs. Geotextile bonded 1.566, jointed 1.559: the clay squeezes out under the embankment and the sheet is stretched across it to capacity in both. Liner bonded 2.167, jointed 1.285: the bonded model can only fail the fill's faces, the jointed one slides two wedges out on the liner. Both field states are captured for every run; the page shows last converged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_liner_bonded.xlsx
+++ b/docs/tutorials/files/xslope_liner_bonded.xlsx
@@ -8706,7 +8706,7 @@
         </is>
       </c>
       <c r="F12" s="3">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="G12" s="3">
         <v>34.0</v>
@@ -10219,7 +10219,7 @@
         <v>145</v>
       </c>
       <c r="B2" s="3">
-        <v>-5.0</v>
+        <v>-4.0</v>
       </c>
       <c r="D2" s="24" t="s">
         <v>146</v>
@@ -12062,7 +12062,7 @@
         <v>0.0</v>
       </c>
       <c r="B10" s="3">
-        <v>-5.0</v>
+        <v>-4.0</v>
       </c>
       <c r="D10" s="3">
         <v>14.0</v>
@@ -12110,7 +12110,7 @@
         <v>60.0</v>
       </c>
       <c r="B11" s="3">
-        <v>-5.0</v>
+        <v>-4.0</v>
       </c>
       <c r="D11" s="3">
         <v>46.0</v>
@@ -13269,7 +13269,7 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <v>-5.0</v>
+        <v>-4.0</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>

</xml_diff>